<commit_message>
docs: actualizar seguimiento semanal, modelo pedagogico en README, matriz 15 articulos y rectificar actividades
</commit_message>
<xml_diff>
--- a/docs/investigacion/MATRIZ_15_ARTICULOS.xlsx
+++ b/docs/investigacion/MATRIZ_15_ARTICULOS.xlsx
@@ -1,21 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AE290B7-7620-4568-BD51-B63AB9A17DA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Matriz Principal" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Artículos Reemplazados" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Fuentes y Verificación" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="Responsables" state="visible" r:id="rId7"/>
-    <sheet sheetId="5" name="Relación MODESEC" state="visible" r:id="rId8"/>
+    <sheet name="Matriz Principal" sheetId="1" r:id="rId1"/>
+    <sheet name="Artículos Reemplazados" sheetId="2" r:id="rId2"/>
+    <sheet name="Fuentes y Verificación" sheetId="3" r:id="rId3"/>
+    <sheet name="Responsables" sheetId="4" r:id="rId4"/>
+    <sheet name="Relación MODESEC" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="501" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="468" uniqueCount="283">
   <si>
     <t>Nº</t>
   </si>
@@ -71,9 +75,6 @@
     <t>MODESEC</t>
   </si>
   <si>
-    <t>Responsable reportado</t>
-  </si>
-  <si>
     <t>Responsable análisis</t>
   </si>
   <si>
@@ -852,9 +853,6 @@
   </si>
   <si>
     <t>https://doi.org/10.1007/s10209-023-00967-2</t>
-  </si>
-  <si>
-    <t>Responsable Histórico Reportado</t>
   </si>
   <si>
     <t>Responsable de Análisis</t>
@@ -875,17 +873,19 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1249,9 +1249,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:U16"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:T16"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
@@ -1265,11 +1265,11 @@
     <col min="12" max="13" width="20" customWidth="1"/>
     <col min="14" max="17" width="30" customWidth="1"/>
     <col min="18" max="18" width="20" customWidth="1"/>
-    <col min="19" max="20" width="15" customWidth="1"/>
-    <col min="21" max="21" width="10" customWidth="1"/>
+    <col min="19" max="19" width="15" customWidth="1"/>
+    <col min="20" max="20" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1330,64 +1330,61 @@
       <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="B2" t="s">
         <v>21</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>22</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>23</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>24</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>25</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>26</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>27</v>
       </c>
-      <c r="H2" t="s">
-        <v>28</v>
-      </c>
       <c r="I2" t="s">
+        <v>28</v>
+      </c>
+      <c r="J2" t="s">
         <v>29</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>30</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>31</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>32</v>
       </c>
-      <c r="M2" t="s">
+      <c r="N2" t="s">
         <v>33</v>
       </c>
-      <c r="N2" t="s">
+      <c r="O2" t="s">
         <v>34</v>
       </c>
-      <c r="O2" t="s">
+      <c r="P2" t="s">
         <v>35</v>
       </c>
-      <c r="P2" t="s">
+      <c r="Q2" t="s">
         <v>36</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="R2" t="s">
         <v>37</v>
-      </c>
-      <c r="R2" t="s">
-        <v>38</v>
       </c>
       <c r="S2" t="s">
         <v>39</v>
@@ -1395,649 +1392,619 @@
       <c r="T2" t="s">
         <v>40</v>
       </c>
-      <c r="U2" t="s">
+    </row>
+    <row r="3" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="B3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3" t="s">
         <v>42</v>
       </c>
-      <c r="B3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>43</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>44</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>45</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>46</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>47</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
+        <v>28</v>
+      </c>
+      <c r="J3" t="s">
         <v>48</v>
       </c>
-      <c r="I3" t="s">
-        <v>29</v>
-      </c>
-      <c r="J3" t="s">
+      <c r="K3" t="s">
         <v>49</v>
       </c>
-      <c r="K3" t="s">
+      <c r="L3" t="s">
         <v>50</v>
       </c>
-      <c r="L3" t="s">
+      <c r="M3" t="s">
         <v>51</v>
       </c>
-      <c r="M3" t="s">
+      <c r="N3" t="s">
         <v>52</v>
       </c>
-      <c r="N3" t="s">
+      <c r="O3" t="s">
         <v>53</v>
       </c>
-      <c r="O3" t="s">
+      <c r="P3" t="s">
         <v>54</v>
       </c>
-      <c r="P3" t="s">
+      <c r="Q3" t="s">
         <v>55</v>
       </c>
-      <c r="Q3" t="s">
+      <c r="R3" t="s">
         <v>56</v>
       </c>
-      <c r="R3" t="s">
+      <c r="S3" t="s">
         <v>57</v>
       </c>
-      <c r="S3" t="s">
-        <v>39</v>
-      </c>
       <c r="T3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>58</v>
       </c>
-      <c r="U3" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="B4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" t="s">
         <v>59</v>
       </c>
-      <c r="B4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>60</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>61</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>62</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>63</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
+        <v>27</v>
+      </c>
+      <c r="I4" t="s">
+        <v>28</v>
+      </c>
+      <c r="J4" t="s">
         <v>64</v>
       </c>
-      <c r="H4" t="s">
-        <v>28</v>
-      </c>
-      <c r="I4" t="s">
-        <v>29</v>
-      </c>
-      <c r="J4" t="s">
+      <c r="K4" t="s">
         <v>65</v>
       </c>
-      <c r="K4" t="s">
+      <c r="L4" t="s">
         <v>66</v>
       </c>
-      <c r="L4" t="s">
+      <c r="M4" t="s">
         <v>67</v>
       </c>
-      <c r="M4" t="s">
+      <c r="N4" t="s">
         <v>68</v>
       </c>
-      <c r="N4" t="s">
+      <c r="O4" t="s">
         <v>69</v>
       </c>
-      <c r="O4" t="s">
+      <c r="P4" t="s">
         <v>70</v>
       </c>
-      <c r="P4" t="s">
+      <c r="Q4" t="s">
         <v>71</v>
       </c>
-      <c r="Q4" t="s">
+      <c r="R4" t="s">
         <v>72</v>
       </c>
-      <c r="R4" t="s">
+      <c r="S4" t="s">
+        <v>38</v>
+      </c>
+      <c r="T4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
         <v>73</v>
       </c>
-      <c r="S4" t="s">
-        <v>39</v>
-      </c>
-      <c r="T4" t="s">
-        <v>39</v>
-      </c>
-      <c r="U4" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="B5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" t="s">
         <v>74</v>
       </c>
-      <c r="B5" t="s">
-        <v>22</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>75</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>76</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>77</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>78</v>
       </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
+        <v>47</v>
+      </c>
+      <c r="I5" t="s">
+        <v>28</v>
+      </c>
+      <c r="J5" t="s">
         <v>79</v>
       </c>
-      <c r="H5" t="s">
-        <v>48</v>
-      </c>
-      <c r="I5" t="s">
-        <v>29</v>
-      </c>
-      <c r="J5" t="s">
+      <c r="K5" t="s">
         <v>80</v>
       </c>
-      <c r="K5" t="s">
+      <c r="L5" t="s">
         <v>81</v>
       </c>
-      <c r="L5" t="s">
+      <c r="M5" t="s">
         <v>82</v>
       </c>
-      <c r="M5" t="s">
+      <c r="N5" t="s">
         <v>83</v>
       </c>
-      <c r="N5" t="s">
+      <c r="O5" t="s">
         <v>84</v>
       </c>
-      <c r="O5" t="s">
+      <c r="P5" t="s">
         <v>85</v>
       </c>
-      <c r="P5" t="s">
+      <c r="Q5" t="s">
         <v>86</v>
       </c>
-      <c r="Q5" t="s">
+      <c r="R5" t="s">
         <v>87</v>
       </c>
-      <c r="R5" t="s">
+      <c r="S5" t="s">
         <v>88</v>
       </c>
-      <c r="S5" t="s">
-        <v>39</v>
-      </c>
       <c r="T5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
         <v>89</v>
       </c>
-      <c r="U5" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="B6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" t="s">
         <v>90</v>
       </c>
-      <c r="B6" t="s">
-        <v>22</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>91</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>92</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>93</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>94</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>95</v>
       </c>
-      <c r="H6" t="s">
+      <c r="I6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J6" t="s">
         <v>96</v>
       </c>
-      <c r="I6" t="s">
-        <v>29</v>
-      </c>
-      <c r="J6" t="s">
+      <c r="K6" t="s">
         <v>97</v>
       </c>
-      <c r="K6" t="s">
+      <c r="L6" t="s">
+        <v>66</v>
+      </c>
+      <c r="M6" t="s">
         <v>98</v>
       </c>
-      <c r="L6" t="s">
-        <v>67</v>
-      </c>
-      <c r="M6" t="s">
+      <c r="N6" t="s">
         <v>99</v>
       </c>
-      <c r="N6" t="s">
+      <c r="O6" t="s">
         <v>100</v>
       </c>
-      <c r="O6" t="s">
+      <c r="P6" t="s">
         <v>101</v>
       </c>
-      <c r="P6" t="s">
+      <c r="Q6" t="s">
         <v>102</v>
       </c>
-      <c r="Q6" t="s">
+      <c r="R6" t="s">
         <v>103</v>
       </c>
-      <c r="R6" t="s">
+      <c r="S6" t="s">
         <v>104</v>
       </c>
-      <c r="S6" t="s">
-        <v>39</v>
-      </c>
       <c r="T6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
         <v>105</v>
       </c>
-      <c r="U6" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="B7" t="s">
         <v>106</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>107</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>108</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>109</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>110</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>111</v>
       </c>
-      <c r="G7" t="s">
+      <c r="H7" t="s">
         <v>112</v>
       </c>
-      <c r="H7" t="s">
+      <c r="I7" t="s">
+        <v>28</v>
+      </c>
+      <c r="J7" t="s">
         <v>113</v>
       </c>
-      <c r="I7" t="s">
-        <v>29</v>
-      </c>
-      <c r="J7" t="s">
+      <c r="K7" t="s">
         <v>114</v>
       </c>
-      <c r="K7" t="s">
+      <c r="L7" t="s">
         <v>115</v>
       </c>
-      <c r="L7" t="s">
+      <c r="M7" t="s">
         <v>116</v>
       </c>
-      <c r="M7" t="s">
+      <c r="N7" t="s">
         <v>117</v>
       </c>
-      <c r="N7" t="s">
+      <c r="O7" t="s">
         <v>118</v>
       </c>
-      <c r="O7" t="s">
+      <c r="P7" t="s">
         <v>119</v>
       </c>
-      <c r="P7" t="s">
+      <c r="Q7" t="s">
         <v>120</v>
       </c>
-      <c r="Q7" t="s">
+      <c r="R7" t="s">
         <v>121</v>
       </c>
-      <c r="R7" t="s">
+      <c r="S7" t="s">
+        <v>57</v>
+      </c>
+      <c r="T7" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
         <v>122</v>
       </c>
-      <c r="S7" t="s">
-        <v>39</v>
-      </c>
-      <c r="T7" t="s">
-        <v>58</v>
-      </c>
-      <c r="U7" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="B8" t="s">
+        <v>106</v>
+      </c>
+      <c r="C8" t="s">
         <v>123</v>
       </c>
-      <c r="B8" t="s">
-        <v>107</v>
-      </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>124</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
+        <v>109</v>
+      </c>
+      <c r="F8" t="s">
         <v>125</v>
       </c>
-      <c r="E8" t="s">
-        <v>110</v>
-      </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
         <v>126</v>
       </c>
-      <c r="G8" t="s">
+      <c r="H8" t="s">
         <v>127</v>
       </c>
-      <c r="H8" t="s">
+      <c r="I8" t="s">
+        <v>28</v>
+      </c>
+      <c r="J8" t="s">
         <v>128</v>
       </c>
-      <c r="I8" t="s">
-        <v>29</v>
-      </c>
-      <c r="J8" t="s">
+      <c r="K8" t="s">
         <v>129</v>
       </c>
-      <c r="K8" t="s">
+      <c r="L8" t="s">
         <v>130</v>
       </c>
-      <c r="L8" t="s">
+      <c r="M8" t="s">
         <v>131</v>
       </c>
-      <c r="M8" t="s">
+      <c r="N8" t="s">
         <v>132</v>
       </c>
-      <c r="N8" t="s">
+      <c r="O8" t="s">
         <v>133</v>
       </c>
-      <c r="O8" t="s">
+      <c r="P8" t="s">
         <v>134</v>
       </c>
-      <c r="P8" t="s">
+      <c r="Q8" t="s">
         <v>135</v>
       </c>
-      <c r="Q8" t="s">
+      <c r="R8" t="s">
+        <v>121</v>
+      </c>
+      <c r="S8" t="s">
+        <v>88</v>
+      </c>
+      <c r="T8" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
         <v>136</v>
       </c>
-      <c r="R8" t="s">
-        <v>122</v>
-      </c>
-      <c r="S8" t="s">
-        <v>39</v>
-      </c>
-      <c r="T8" t="s">
-        <v>89</v>
-      </c>
-      <c r="U8" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="B9" t="s">
+        <v>106</v>
+      </c>
+      <c r="C9" t="s">
         <v>137</v>
       </c>
-      <c r="B9" t="s">
-        <v>107</v>
-      </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>138</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
+        <v>44</v>
+      </c>
+      <c r="F9" t="s">
         <v>139</v>
       </c>
-      <c r="E9" t="s">
-        <v>45</v>
-      </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
         <v>140</v>
       </c>
-      <c r="G9" t="s">
+      <c r="H9" t="s">
+        <v>47</v>
+      </c>
+      <c r="I9" t="s">
+        <v>28</v>
+      </c>
+      <c r="J9" t="s">
         <v>141</v>
       </c>
-      <c r="H9" t="s">
-        <v>48</v>
-      </c>
-      <c r="I9" t="s">
-        <v>29</v>
-      </c>
-      <c r="J9" t="s">
+      <c r="K9" t="s">
         <v>142</v>
       </c>
-      <c r="K9" t="s">
+      <c r="L9" t="s">
         <v>143</v>
       </c>
-      <c r="L9" t="s">
+      <c r="M9" t="s">
         <v>144</v>
       </c>
-      <c r="M9" t="s">
+      <c r="N9" t="s">
         <v>145</v>
       </c>
-      <c r="N9" t="s">
+      <c r="O9" t="s">
         <v>146</v>
       </c>
-      <c r="O9" t="s">
+      <c r="P9" t="s">
         <v>147</v>
       </c>
-      <c r="P9" t="s">
+      <c r="Q9" t="s">
         <v>148</v>
       </c>
-      <c r="Q9" t="s">
+      <c r="R9" t="s">
         <v>149</v>
       </c>
-      <c r="R9" t="s">
+      <c r="S9" t="s">
+        <v>38</v>
+      </c>
+      <c r="T9" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="10" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
         <v>150</v>
       </c>
-      <c r="S9" t="s">
-        <v>39</v>
-      </c>
-      <c r="T9" t="s">
-        <v>39</v>
-      </c>
-      <c r="U9" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="B10" t="s">
+        <v>106</v>
+      </c>
+      <c r="C10" t="s">
         <v>151</v>
       </c>
-      <c r="B10" t="s">
-        <v>107</v>
-      </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
         <v>152</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
+        <v>44</v>
+      </c>
+      <c r="F10" t="s">
         <v>153</v>
       </c>
-      <c r="E10" t="s">
-        <v>45</v>
-      </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
         <v>154</v>
       </c>
-      <c r="G10" t="s">
+      <c r="H10" t="s">
         <v>155</v>
       </c>
-      <c r="H10" t="s">
+      <c r="I10" t="s">
+        <v>28</v>
+      </c>
+      <c r="J10" t="s">
         <v>156</v>
       </c>
-      <c r="I10" t="s">
-        <v>29</v>
-      </c>
-      <c r="J10" t="s">
+      <c r="K10" t="s">
         <v>157</v>
       </c>
-      <c r="K10" t="s">
+      <c r="L10" t="s">
         <v>158</v>
       </c>
-      <c r="L10" t="s">
+      <c r="M10" t="s">
         <v>159</v>
       </c>
-      <c r="M10" t="s">
+      <c r="N10" t="s">
         <v>160</v>
       </c>
-      <c r="N10" t="s">
+      <c r="O10" t="s">
         <v>161</v>
       </c>
-      <c r="O10" t="s">
+      <c r="P10" t="s">
         <v>162</v>
       </c>
-      <c r="P10" t="s">
+      <c r="Q10" t="s">
         <v>163</v>
       </c>
-      <c r="Q10" t="s">
+      <c r="R10" t="s">
+        <v>121</v>
+      </c>
+      <c r="S10" t="s">
+        <v>104</v>
+      </c>
+      <c r="T10" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="11" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
         <v>164</v>
       </c>
-      <c r="R10" t="s">
-        <v>122</v>
-      </c>
-      <c r="S10" t="s">
-        <v>39</v>
-      </c>
-      <c r="T10" t="s">
-        <v>105</v>
-      </c>
-      <c r="U10" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="B11" t="s">
+        <v>106</v>
+      </c>
+      <c r="C11" t="s">
         <v>165</v>
       </c>
-      <c r="B11" t="s">
-        <v>107</v>
-      </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
         <v>166</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
+        <v>76</v>
+      </c>
+      <c r="F11" t="s">
         <v>167</v>
       </c>
-      <c r="E11" t="s">
-        <v>77</v>
-      </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
         <v>168</v>
       </c>
-      <c r="G11" t="s">
+      <c r="H11" t="s">
         <v>169</v>
       </c>
-      <c r="H11" t="s">
+      <c r="I11" t="s">
+        <v>28</v>
+      </c>
+      <c r="J11" t="s">
         <v>170</v>
       </c>
-      <c r="I11" t="s">
-        <v>29</v>
-      </c>
-      <c r="J11" t="s">
+      <c r="K11" t="s">
         <v>171</v>
       </c>
-      <c r="K11" t="s">
+      <c r="L11" t="s">
         <v>172</v>
       </c>
-      <c r="L11" t="s">
+      <c r="M11" t="s">
         <v>173</v>
       </c>
-      <c r="M11" t="s">
+      <c r="N11" t="s">
         <v>174</v>
       </c>
-      <c r="N11" t="s">
+      <c r="O11" t="s">
         <v>175</v>
       </c>
-      <c r="O11" t="s">
+      <c r="P11" t="s">
         <v>176</v>
       </c>
-      <c r="P11" t="s">
+      <c r="Q11" t="s">
         <v>177</v>
       </c>
-      <c r="Q11" t="s">
+      <c r="R11" t="s">
         <v>178</v>
       </c>
-      <c r="R11" t="s">
+      <c r="S11" t="s">
         <v>179</v>
       </c>
-      <c r="S11" t="s">
-        <v>39</v>
-      </c>
       <c r="T11" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
         <v>180</v>
       </c>
-      <c r="U11" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+      <c r="B12" t="s">
         <v>181</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
         <v>182</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
         <v>183</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
+        <v>44</v>
+      </c>
+      <c r="F12" t="s">
         <v>184</v>
       </c>
-      <c r="E12" t="s">
-        <v>45</v>
-      </c>
-      <c r="F12" t="s">
+      <c r="G12" t="s">
         <v>185</v>
       </c>
-      <c r="G12" t="s">
+      <c r="H12" t="s">
+        <v>127</v>
+      </c>
+      <c r="I12" t="s">
+        <v>28</v>
+      </c>
+      <c r="J12" t="s">
         <v>186</v>
       </c>
-      <c r="H12" t="s">
-        <v>128</v>
-      </c>
-      <c r="I12" t="s">
-        <v>29</v>
-      </c>
-      <c r="J12" t="s">
+      <c r="K12" t="s">
         <v>187</v>
       </c>
-      <c r="K12" t="s">
+      <c r="L12" t="s">
         <v>188</v>
       </c>
-      <c r="L12" t="s">
+      <c r="M12" t="s">
         <v>189</v>
       </c>
-      <c r="M12" t="s">
+      <c r="N12" t="s">
         <v>190</v>
       </c>
-      <c r="N12" t="s">
+      <c r="O12" t="s">
         <v>191</v>
       </c>
-      <c r="O12" t="s">
+      <c r="P12" t="s">
         <v>192</v>
       </c>
-      <c r="P12" t="s">
+      <c r="Q12" t="s">
         <v>193</v>
       </c>
-      <c r="Q12" t="s">
+      <c r="R12" t="s">
         <v>194</v>
-      </c>
-      <c r="R12" t="s">
-        <v>195</v>
       </c>
       <c r="S12" t="s">
         <v>39</v>
@@ -2045,280 +2012,265 @@
       <c r="T12" t="s">
         <v>40</v>
       </c>
-      <c r="U12" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
+        <v>195</v>
+      </c>
+      <c r="B13" t="s">
+        <v>181</v>
+      </c>
+      <c r="C13" t="s">
         <v>196</v>
       </c>
-      <c r="B13" t="s">
-        <v>182</v>
-      </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>197</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
+        <v>24</v>
+      </c>
+      <c r="F13" t="s">
         <v>198</v>
       </c>
-      <c r="E13" t="s">
-        <v>25</v>
-      </c>
-      <c r="F13" t="s">
+      <c r="G13" t="s">
         <v>199</v>
       </c>
-      <c r="G13" t="s">
+      <c r="H13" t="s">
+        <v>95</v>
+      </c>
+      <c r="I13" t="s">
+        <v>28</v>
+      </c>
+      <c r="J13" t="s">
         <v>200</v>
       </c>
-      <c r="H13" t="s">
-        <v>96</v>
-      </c>
-      <c r="I13" t="s">
-        <v>29</v>
-      </c>
-      <c r="J13" t="s">
+      <c r="K13" t="s">
         <v>201</v>
       </c>
-      <c r="K13" t="s">
+      <c r="L13" t="s">
         <v>202</v>
       </c>
-      <c r="L13" t="s">
+      <c r="M13" t="s">
         <v>203</v>
       </c>
-      <c r="M13" t="s">
+      <c r="N13" t="s">
         <v>204</v>
       </c>
-      <c r="N13" t="s">
+      <c r="O13" t="s">
         <v>205</v>
       </c>
-      <c r="O13" t="s">
+      <c r="P13" t="s">
         <v>206</v>
       </c>
-      <c r="P13" t="s">
+      <c r="Q13" t="s">
         <v>207</v>
       </c>
-      <c r="Q13" t="s">
+      <c r="R13" t="s">
+        <v>194</v>
+      </c>
+      <c r="S13" t="s">
+        <v>57</v>
+      </c>
+      <c r="T13" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="14" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
         <v>208</v>
       </c>
-      <c r="R13" t="s">
-        <v>195</v>
-      </c>
-      <c r="S13" t="s">
-        <v>39</v>
-      </c>
-      <c r="T13" t="s">
-        <v>58</v>
-      </c>
-      <c r="U13" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+      <c r="B14" t="s">
+        <v>181</v>
+      </c>
+      <c r="C14" t="s">
         <v>209</v>
       </c>
-      <c r="B14" t="s">
-        <v>182</v>
-      </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
         <v>210</v>
       </c>
-      <c r="D14" t="s">
+      <c r="E14" t="s">
+        <v>76</v>
+      </c>
+      <c r="F14" t="s">
         <v>211</v>
       </c>
-      <c r="E14" t="s">
-        <v>77</v>
-      </c>
-      <c r="F14" t="s">
+      <c r="G14" t="s">
         <v>212</v>
       </c>
-      <c r="G14" t="s">
+      <c r="H14" t="s">
+        <v>155</v>
+      </c>
+      <c r="I14" t="s">
+        <v>28</v>
+      </c>
+      <c r="J14" t="s">
         <v>213</v>
       </c>
-      <c r="H14" t="s">
-        <v>156</v>
-      </c>
-      <c r="I14" t="s">
-        <v>29</v>
-      </c>
-      <c r="J14" t="s">
+      <c r="K14" t="s">
         <v>214</v>
       </c>
-      <c r="K14" t="s">
+      <c r="L14" t="s">
         <v>215</v>
       </c>
-      <c r="L14" t="s">
+      <c r="M14" t="s">
         <v>216</v>
       </c>
-      <c r="M14" t="s">
+      <c r="N14" t="s">
         <v>217</v>
       </c>
-      <c r="N14" t="s">
+      <c r="O14" t="s">
         <v>218</v>
       </c>
-      <c r="O14" t="s">
+      <c r="P14" t="s">
         <v>219</v>
       </c>
-      <c r="P14" t="s">
+      <c r="Q14" t="s">
         <v>220</v>
       </c>
-      <c r="Q14" t="s">
+      <c r="R14" t="s">
+        <v>194</v>
+      </c>
+      <c r="S14" t="s">
+        <v>179</v>
+      </c>
+      <c r="T14" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="15" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
         <v>221</v>
       </c>
-      <c r="R14" t="s">
-        <v>195</v>
-      </c>
-      <c r="S14" t="s">
-        <v>39</v>
-      </c>
-      <c r="T14" t="s">
-        <v>180</v>
-      </c>
-      <c r="U14" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+      <c r="B15" t="s">
+        <v>181</v>
+      </c>
+      <c r="C15" t="s">
         <v>222</v>
       </c>
-      <c r="B15" t="s">
-        <v>182</v>
-      </c>
-      <c r="C15" t="s">
+      <c r="D15" t="s">
         <v>223</v>
       </c>
-      <c r="D15" t="s">
+      <c r="E15" t="s">
         <v>224</v>
       </c>
-      <c r="E15" t="s">
+      <c r="F15" t="s">
         <v>225</v>
       </c>
-      <c r="F15" t="s">
+      <c r="G15" t="s">
         <v>226</v>
       </c>
-      <c r="G15" t="s">
+      <c r="H15" t="s">
+        <v>27</v>
+      </c>
+      <c r="I15" t="s">
+        <v>28</v>
+      </c>
+      <c r="J15" t="s">
         <v>227</v>
       </c>
-      <c r="H15" t="s">
-        <v>28</v>
-      </c>
-      <c r="I15" t="s">
-        <v>29</v>
-      </c>
-      <c r="J15" t="s">
+      <c r="K15" t="s">
         <v>228</v>
       </c>
-      <c r="K15" t="s">
+      <c r="L15" t="s">
+        <v>172</v>
+      </c>
+      <c r="M15" t="s">
         <v>229</v>
       </c>
-      <c r="L15" t="s">
-        <v>173</v>
-      </c>
-      <c r="M15" t="s">
+      <c r="N15" t="s">
         <v>230</v>
       </c>
-      <c r="N15" t="s">
+      <c r="O15" t="s">
         <v>231</v>
       </c>
-      <c r="O15" t="s">
+      <c r="P15" t="s">
         <v>232</v>
       </c>
-      <c r="P15" t="s">
+      <c r="Q15" t="s">
         <v>233</v>
       </c>
-      <c r="Q15" t="s">
+      <c r="R15" t="s">
         <v>234</v>
       </c>
-      <c r="R15" t="s">
+      <c r="S15" t="s">
+        <v>38</v>
+      </c>
+      <c r="T15" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="16" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
         <v>235</v>
       </c>
-      <c r="S15" t="s">
-        <v>39</v>
-      </c>
-      <c r="T15" t="s">
-        <v>39</v>
-      </c>
-      <c r="U15" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+      <c r="B16" t="s">
+        <v>181</v>
+      </c>
+      <c r="C16" t="s">
         <v>236</v>
       </c>
-      <c r="B16" t="s">
-        <v>182</v>
-      </c>
-      <c r="C16" t="s">
+      <c r="D16" t="s">
         <v>237</v>
       </c>
-      <c r="D16" t="s">
+      <c r="E16" t="s">
+        <v>44</v>
+      </c>
+      <c r="F16" t="s">
         <v>238</v>
       </c>
-      <c r="E16" t="s">
-        <v>45</v>
-      </c>
-      <c r="F16" t="s">
+      <c r="G16" t="s">
         <v>239</v>
       </c>
-      <c r="G16" t="s">
+      <c r="H16" t="s">
+        <v>47</v>
+      </c>
+      <c r="I16" t="s">
+        <v>28</v>
+      </c>
+      <c r="J16" t="s">
         <v>240</v>
       </c>
-      <c r="H16" t="s">
-        <v>48</v>
-      </c>
-      <c r="I16" t="s">
-        <v>29</v>
-      </c>
-      <c r="J16" t="s">
+      <c r="K16" t="s">
         <v>241</v>
       </c>
-      <c r="K16" t="s">
+      <c r="L16" t="s">
         <v>242</v>
       </c>
-      <c r="L16" t="s">
+      <c r="M16" t="s">
         <v>243</v>
       </c>
-      <c r="M16" t="s">
+      <c r="N16" t="s">
         <v>244</v>
       </c>
-      <c r="N16" t="s">
+      <c r="O16" t="s">
         <v>245</v>
       </c>
-      <c r="O16" t="s">
+      <c r="P16" t="s">
         <v>246</v>
       </c>
-      <c r="P16" t="s">
+      <c r="Q16" t="s">
         <v>247</v>
       </c>
-      <c r="Q16" t="s">
-        <v>248</v>
-      </c>
       <c r="R16" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="S16" t="s">
-        <v>39</v>
+        <v>88</v>
       </c>
       <c r="T16" t="s">
-        <v>89</v>
-      </c>
-      <c r="U16" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
     <col min="2" max="2" width="25" customWidth="1"/>
@@ -2326,72 +2278,72 @@
     <col min="4" max="4" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>250</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="B2" t="s">
         <v>251</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>252</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>253</v>
       </c>
-      <c r="D2" t="s">
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>254</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="B3" t="s">
         <v>255</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>256</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>257</v>
       </c>
-      <c r="D3" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="B4" t="s">
         <v>258</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>259</v>
       </c>
-      <c r="C4" t="s">
-        <v>260</v>
-      </c>
       <c r="D4" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D16"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="40" customWidth="1"/>
@@ -2399,584 +2351,533 @@
     <col min="4" max="4" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>261</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>262</v>
       </c>
-      <c r="D1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" t="s">
         <v>264</v>
       </c>
-      <c r="C2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>42</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>58</v>
+      </c>
+      <c r="B4" t="s">
         <v>265</v>
       </c>
-      <c r="C3" t="s">
-        <v>48</v>
-      </c>
-      <c r="D3" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>59</v>
-      </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>73</v>
+      </c>
+      <c r="B5" t="s">
         <v>266</v>
       </c>
-      <c r="C4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D4" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>74</v>
-      </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
+        <v>47</v>
+      </c>
+      <c r="D5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>89</v>
+      </c>
+      <c r="B6" t="s">
         <v>267</v>
       </c>
-      <c r="C5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>90</v>
-      </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
+        <v>95</v>
+      </c>
+      <c r="D6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>105</v>
+      </c>
+      <c r="B7" t="s">
         <v>268</v>
       </c>
-      <c r="C6" t="s">
-        <v>96</v>
-      </c>
-      <c r="D6" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>106</v>
-      </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
+        <v>112</v>
+      </c>
+      <c r="D7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>122</v>
+      </c>
+      <c r="B8" t="s">
         <v>269</v>
       </c>
-      <c r="C7" t="s">
-        <v>113</v>
-      </c>
-      <c r="D7" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>123</v>
-      </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
+        <v>127</v>
+      </c>
+      <c r="D8" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>136</v>
+      </c>
+      <c r="B9" t="s">
         <v>270</v>
       </c>
-      <c r="C8" t="s">
-        <v>128</v>
-      </c>
-      <c r="D8" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>137</v>
-      </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
+        <v>47</v>
+      </c>
+      <c r="D9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>150</v>
+      </c>
+      <c r="B10" t="s">
         <v>271</v>
       </c>
-      <c r="C9" t="s">
-        <v>48</v>
-      </c>
-      <c r="D9" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>151</v>
-      </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
+        <v>155</v>
+      </c>
+      <c r="D10" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>164</v>
+      </c>
+      <c r="B11" t="s">
         <v>272</v>
       </c>
-      <c r="C10" t="s">
-        <v>156</v>
-      </c>
-      <c r="D10" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>165</v>
-      </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
+        <v>169</v>
+      </c>
+      <c r="D11" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>180</v>
+      </c>
+      <c r="B12" t="s">
         <v>273</v>
       </c>
-      <c r="C11" t="s">
-        <v>170</v>
-      </c>
-      <c r="D11" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>181</v>
-      </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
+        <v>127</v>
+      </c>
+      <c r="D12" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>195</v>
+      </c>
+      <c r="B13" t="s">
         <v>274</v>
       </c>
-      <c r="C12" t="s">
-        <v>128</v>
-      </c>
-      <c r="D12" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>196</v>
-      </c>
-      <c r="B13" t="s">
+      <c r="C13" t="s">
+        <v>95</v>
+      </c>
+      <c r="D13" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>208</v>
+      </c>
+      <c r="B14" t="s">
         <v>275</v>
       </c>
-      <c r="C13" t="s">
-        <v>96</v>
-      </c>
-      <c r="D13" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>209</v>
-      </c>
-      <c r="B14" t="s">
+      <c r="C14" t="s">
+        <v>155</v>
+      </c>
+      <c r="D14" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>221</v>
+      </c>
+      <c r="B15" t="s">
         <v>276</v>
       </c>
-      <c r="C14" t="s">
-        <v>156</v>
-      </c>
-      <c r="D14" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>222</v>
-      </c>
-      <c r="B15" t="s">
+      <c r="C15" t="s">
+        <v>27</v>
+      </c>
+      <c r="D15" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>235</v>
+      </c>
+      <c r="B16" t="s">
         <v>277</v>
       </c>
-      <c r="C15" t="s">
-        <v>28</v>
-      </c>
-      <c r="D15" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>236</v>
-      </c>
-      <c r="B16" t="s">
-        <v>278</v>
-      </c>
       <c r="C16" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D16" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D17"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
-    <col min="2" max="3" width="30" customWidth="1"/>
-    <col min="4" max="4" width="40" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="3" max="3" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>279</v>
       </c>
-      <c r="C1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>280</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="B2" t="s">
+        <v>280</v>
+      </c>
+      <c r="C2" t="s">
         <v>281</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>282</v>
-      </c>
-      <c r="B2" t="s">
-        <v>282</v>
-      </c>
-      <c r="C2" t="s">
-        <v>282</v>
-      </c>
-      <c r="D2" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B3" t="s">
         <v>39</v>
       </c>
-      <c r="C3" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B4" t="s">
-        <v>39</v>
-      </c>
-      <c r="C4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>59</v>
-      </c>
       <c r="B5" t="s">
-        <v>39</v>
-      </c>
-      <c r="C5" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B6" t="s">
-        <v>39</v>
-      </c>
-      <c r="C6" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>90</v>
-      </c>
       <c r="B7" t="s">
-        <v>39</v>
-      </c>
-      <c r="C7" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>106</v>
-      </c>
       <c r="B8" t="s">
-        <v>39</v>
-      </c>
-      <c r="C8" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B9" t="s">
-        <v>39</v>
-      </c>
-      <c r="C9" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B10" t="s">
-        <v>39</v>
-      </c>
-      <c r="C10" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B11" t="s">
-        <v>39</v>
-      </c>
-      <c r="C11" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B12" t="s">
-        <v>39</v>
-      </c>
-      <c r="C12" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
         <v>180</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>181</v>
       </c>
       <c r="B13" t="s">
         <v>39</v>
       </c>
-      <c r="C13" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B14" t="s">
-        <v>39</v>
-      </c>
-      <c r="C14" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B15" t="s">
-        <v>39</v>
-      </c>
-      <c r="C15" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B16" t="s">
-        <v>39</v>
-      </c>
-      <c r="C16" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B17" t="s">
-        <v>39</v>
-      </c>
-      <c r="C17" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:B16"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B2" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B3" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B4" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>74</v>
-      </c>
       <c r="B5" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B6" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B7" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>123</v>
-      </c>
       <c r="B8" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B9" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>151</v>
-      </c>
       <c r="B10" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B11" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B12" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>196</v>
-      </c>
       <c r="B13" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B14" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B15" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
         <v>235</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>236</v>
-      </c>
       <c r="B16" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>